<commit_message>
correccion en devengado del capitulo 5000
</commit_message>
<xml_diff>
--- a/public/CuentasCuentas/5000-Devengado-CuentasCuentasSeguidas.xlsx
+++ b/public/CuentasCuentas/5000-Devengado-CuentasCuentasSeguidas.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\SAC-IPE\public\CuentasCuentas\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\SAC-IPE\public\Guia\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A203FF43-DE19-4896-93E0-68F6669B806A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44C1EB52-6A27-49CD-A235-638F9DC862E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{BA794CD9-A794-4D6D-97A5-04484BD59B08}"/>
   </bookViews>
@@ -1275,12 +1275,18 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
   </fills>
   <borders count="2">
@@ -1310,7 +1316,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1332,6 +1338,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -16315,17 +16327,17 @@
         <v>16</v>
       </c>
     </row>
-    <row r="1048" spans="1:4" ht="60" x14ac:dyDescent="0.25">
-      <c r="A1048" s="4" t="s">
+    <row r="1048" spans="1:4" s="9" customFormat="1" ht="60" x14ac:dyDescent="0.25">
+      <c r="A1048" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="B1048" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="C1048" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="D1048" s="3" t="s">
+      <c r="B1048" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1048" s="8" t="s">
+        <v>7</v>
+      </c>
+      <c r="D1048" s="9" t="s">
         <v>5</v>
       </c>
     </row>
@@ -16686,8 +16698,8 @@
       <c r="B1074" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C1074" s="4" t="s">
-        <v>7</v>
+      <c r="C1074" s="7" t="s">
+        <v>69</v>
       </c>
       <c r="D1074" s="3" t="s">
         <v>5</v>
@@ -16700,8 +16712,8 @@
       <c r="B1075" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C1075" s="4" t="s">
-        <v>7</v>
+      <c r="C1075" s="7" t="s">
+        <v>69</v>
       </c>
       <c r="D1075" s="3" t="s">
         <v>11</v>
@@ -16714,8 +16726,8 @@
       <c r="B1076" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C1076" s="4" t="s">
-        <v>7</v>
+      <c r="C1076" s="7" t="s">
+        <v>69</v>
       </c>
       <c r="D1076" s="3" t="s">
         <v>5</v>
@@ -16728,8 +16740,8 @@
       <c r="B1077" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C1077" s="4" t="s">
-        <v>7</v>
+      <c r="C1077" s="7" t="s">
+        <v>69</v>
       </c>
       <c r="D1077" s="3" t="s">
         <v>11</v>
@@ -16742,8 +16754,8 @@
       <c r="B1078" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C1078" s="4" t="s">
-        <v>7</v>
+      <c r="C1078" s="7" t="s">
+        <v>69</v>
       </c>
       <c r="D1078" s="3" t="s">
         <v>5</v>
@@ -16756,8 +16768,8 @@
       <c r="B1079" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C1079" s="4" t="s">
-        <v>7</v>
+      <c r="C1079" s="7" t="s">
+        <v>69</v>
       </c>
       <c r="D1079" s="3" t="s">
         <v>11</v>
@@ -16770,8 +16782,8 @@
       <c r="B1080" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C1080" s="4" t="s">
-        <v>7</v>
+      <c r="C1080" s="7" t="s">
+        <v>69</v>
       </c>
       <c r="D1080" s="3" t="s">
         <v>5</v>
@@ -16784,8 +16796,8 @@
       <c r="B1081" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="C1081" s="4" t="s">
-        <v>7</v>
+      <c r="C1081" s="7" t="s">
+        <v>69</v>
       </c>
       <c r="D1081" s="3" t="s">
         <v>11</v>

</xml_diff>